<commit_message>
login/otp/bypass/dashboard test cases added
</commit_message>
<xml_diff>
--- a/CP_UI_Automation_Test_Cases.xlsx
+++ b/CP_UI_Automation_Test_Cases.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Login Left Component" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Login" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="OTP Verification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bypass Authentication" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -965,7 +966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1065,7 +1066,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>URL = BASE_URL/ and title matches UAT title</t>
+          <t>URL = BASE_URL/ and title contains 'GrayQuest Education Finance'</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -1076,7 +1077,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Tab title confirmed from live UAT 2026-04-21</t>
+          <t>Asserts title contains 'GrayQuest Education Finance' (Should Contain — resilient to title prefix changes)</t>
         </is>
       </c>
     </row>
@@ -1743,6 +1744,278 @@
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-221</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Login Form Title Is Visible</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>login, ui, title</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Login form should display the title 'What is your Mobile Number?' via data-testid='desktop-view-form-title'.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Title = 'What is your Mobile Number?'</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-222</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Input Note Text Is Visible</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>login, ui, note</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>When no validation error, note below mobile input: 'Please enter the mobile number which you generally use for your banking purposes.'</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>data-testid='mobile-number-input-note' visible and contains note text</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="55" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-223</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Terms Of Service Link In Consent Opens New Tab</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>login, ui, consent, navigation</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>The 'Terms of Services' link inside the consent label should open the T&amp;C page in a new tab.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>New tab title contains 'Terms'</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="55" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-224</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Privacy Policy Link In Consent Opens New Tab</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>login, ui, consent, navigation</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>The 'Privacy Policy' link inside the consent label should open the Privacy Policy page in a new tab.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>New tab title contains 'Privacy'</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="55" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-225</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Number Prefill Via Query Param Navigates To OTP Page</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>login, valid, query-param</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Navigating to /?m=&lt;mobile&gt; pre-fills the mobile field, auto-checks consent, auto-submits, and redirects to /verify.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>URL contains /verify</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>9876543227</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-226</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Footer Is Present On Login Page</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>login, ui, mobile-footer</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>MobileFooter component (data-testid='mobile-footer-container') should be present in the DOM on the login page.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>data-testid='mobile-footer-container' attached in DOM</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Asserts 'attached' state — element is CSS-hidden on desktop viewport</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1756,7 +2029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2312,62 +2585,66 @@
       <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="55" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>TC-311</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>OTP Not Received</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-314</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>OTP With Non-Numeric Characters Shows Error</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>OTP Verification</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>otp, manual, robot:skip</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Manual test — verify UX when OTP is not received (carrier issues).</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>N/A — manual verification</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Cannot automate — requires external SMS gateway dependency</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>otp, validation, negative</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Entering non-numeric characters (e.g. 'abcd') into the OTP field triggers Yup .matches(Regex.otp) validation.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>'Only numeric values allowed'</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>9876543226 / OTP: abcd</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Input has inputMode='numeric' but type='text' — desktop keyboards can type letters</t>
         </is>
       </c>
     </row>
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>TC-312</t>
+          <t>TC-311</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>OTP Timer Disabled State</t>
+          <t>OTP Not Received</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2387,7 +2664,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Manual test — verify timer appearance before countdown starts.</t>
+          <t>Manual test — verify UX when OTP is not received (carrier issues).</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -2403,19 +2680,19 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Cannot reliably automate within normal timing constraints</t>
+          <t>Cannot automate — requires external SMS gateway dependency</t>
         </is>
       </c>
     </row>
     <row r="14" ht="55" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>TC-313</t>
+          <t>TC-312</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Resend OTP After Timer Expires</t>
+          <t>OTP Timer Disabled State</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2425,22 +2702,22 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>otp, slow, resend, robot:skip</t>
+          <t>otp, manual, robot:skip</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Slow / Manual</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>After 180s countdown, Resend OTP link becomes visible. Clicking resets timer.</t>
+          <t>Manual test — verify timer appearance before countdown starts.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Resend link visible after 180s; timer resets after click</t>
+          <t>N/A — manual verification</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
@@ -2450,6 +2727,54 @@
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Cannot reliably automate within normal timing constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>TC-313</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Resend OTP After Timer Expires</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>OTP Verification</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>otp, slow, resend, robot:skip</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Slow / Manual</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>After 180s countdown, Resend OTP link becomes visible. Clicking resets timer.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Resend link visible after 180s; timer resets after click</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>~3 min wait. Run with: robot --include resend tests/otp_tests.robot</t>
         </is>
@@ -2463,11 +2788,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00B6E6CC"/>
+    <tabColor rgb="00F4B8D1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2537,6 +2862,273 @@
     <row r="2" ht="55" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>TC-401</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Bypass Auth With Valid Mobile Redirects Away From Instant Eligibility</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Bypass Authentication</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>bypass-auth, smoke, redirect</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Navigating to /instant-eligibility?m=&lt;valid_mobile&gt; authenticates via bypassAuthPost and redirects away from /instant-eligibility.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>URL no longer contains /instant-eligibility</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-402</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Bypass Auth Without Query Param Redirects To Login Page</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Bypass Authentication</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>bypass-auth, redirect, negative</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Navigating to /instant-eligibility without ?m= redirects to / (login page) with login form visible.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Login form visible; URL does not contain /instant-eligibility</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TC-403</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Bypass Auth No Account Error State Is Visible</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Bypass Authentication</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>bypass-auth, negative, robot:skip</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>When bypassAuthPost fails (mobile has no ERP account), no-account error state should show image and message.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>No-account image and message visible</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Requires UAT mobile that fails bypassAuthPost — not yet identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TC-404</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Sign In Button On No Account State Navigates To Login</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Bypass Authentication</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>bypass-auth, negative, navigation, robot:skip</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>On no-account error state, clicking Sign In should navigate to / (login page).</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Login form visible after Sign In click</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Depends on TC-403 precondition — bypassAuthPost failure state</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00B6E6CC"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Suite</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Test Mobile / Data</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>TC-4001</t>
         </is>
       </c>
@@ -2587,52 +3179,52 @@
       </c>
     </row>
     <row r="3" ht="55" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>TC-4002</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Auto Debit Applications On Dashboard</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>dashboard, auto-debit, robot:skip</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard should display Auto Debit applications.</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Disabled — Auto Debit feature not active in UAT</t>
-        </is>
-      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, auto-debit, tab-navigation</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>The Auto Payments (AD) tab navigation button should be visible on the dashboard.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>data-testid='ad-tab-navigation-button' visible</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>8108556708</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="55" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -2929,12 +3521,12 @@
     <row r="10" ht="55" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TC-4009</t>
+          <t>TC-4032</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Logout Returns To Login Page</t>
+          <t>Insurance Tab Button Is Visible On Dashboard</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2944,22 +3536,22 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>dashboard, profile, logout, session</t>
+          <t>dashboard, insurance, tab-navigation</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Session</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Logout clears auth session and redirects to login page. MUST run last.</t>
+          <t>The Insurance tab navigation button (data-testid='ins-tab-navigation-button') should be visible on the dashboard.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Login form visible after logout</t>
+          <t>Insurance tab button visible</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -2972,21 +3564,17 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>TC-4009 MUST be last test — destroys shared session (TN1 resolution)</t>
-        </is>
-      </c>
+      <c r="J10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="55" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TC-4010</t>
+          <t>TC-4033</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Create New Application Button Has Visible Effect</t>
+          <t>Insurance Tab Click Updates URL Hash</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2996,22 +3584,22 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>dashboard, application, smoke</t>
+          <t>dashboard, insurance, tab-navigation</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Smoke</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Button click produces visible response: modal OR URL change from /my-applications.</t>
+          <t>Clicking the Insurance tab should update the URL hash to #ins and load the Insurance content area.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Modal visible OR URL changed</t>
+          <t>URL contains #ins</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3026,19 +3614,19 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>WARN expected in UAT (no modal — inline form). TN5 dual-branch per O2.</t>
+          <t>InsuranceTab has no data-testid attributes — URL hash is the primary assertion</t>
         </is>
       </c>
     </row>
     <row r="12" ht="55" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TC-4011</t>
+          <t>TC-4009</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>EMI Tab Click Shows EMI Content</t>
+          <t>Logout Returns To Login Page</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -3048,22 +3636,22 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>dashboard, emi, tab-navigation</t>
+          <t>dashboard, profile, logout, session</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Session</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Clicking EMI tab updates URL hash to #emi and shows at least one EMI card.</t>
+          <t>Logout clears auth session and redirects to login page. MUST run last.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>URL contains #emi; EMI card visible</t>
+          <t>Login form visible after logout</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -3078,67 +3666,71 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>PRECONDITION: account must have active EMI applications</t>
+          <t>TC-4009 MUST be last test — destroys shared session (TN1 resolution)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="55" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>TC-4012</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Auto Payments Tab Click</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-4010</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Create New Application Button Has Visible Effect</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>dashboard, auto-payments, robot:skip</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Clicking Auto Payments tab should display Auto Debit content.</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>Disabled — Auto Payments not active in UAT</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, application, smoke</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Button click produces visible response: modal OR URL change from /my-applications.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Modal visible OR URL changed</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>8108556708</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>WARN expected in UAT (no modal — inline form). TN5 dual-branch per O2.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="55" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TC-4013</t>
+          <t>TC-4011</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Transaction History Tab Click</t>
+          <t>EMI Tab Click Shows EMI Content</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -3148,22 +3740,22 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, tab-navigation, smoke</t>
+          <t>dashboard, emi, tab-navigation</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Smoke</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Clicking Transaction History tab updates URL hash to #direct and shows sub-tabs.</t>
+          <t>Clicking EMI tab updates URL hash to #emi and shows at least one EMI card.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>URL contains #direct; Online and Offline sub-tabs visible</t>
+          <t>URL contains #emi; EMI card visible</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -3176,17 +3768,21 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>PRECONDITION: account must have active EMI applications</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-4014</t>
+          <t>TC-4012</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Offline Payments Sub-tab Is Accessible</t>
+          <t>Auto Payments Tab Click</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -3196,7 +3792,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, sub-tab</t>
+          <t>dashboard, auto-payments, tab-navigation</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -3206,12 +3802,12 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Offline Payments sub-tab should be visible and clickable.</t>
+          <t>Clicking the Auto Payments tab button should update the URL hash to #ad and load the Auto Payments content area.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Offline sub-tab clickable</t>
+          <t>URL contains #ad</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -3229,12 +3825,12 @@
     <row r="16" ht="55" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TC-4015</t>
+          <t>TC-4013</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Online Payments Sub-tab Is Accessible</t>
+          <t>Transaction History Tab Click</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -3244,22 +3840,22 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, sub-tab</t>
+          <t>dashboard, pg, tab-navigation, smoke</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Smoke</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Online Payments sub-tab should be visible and clickable.</t>
+          <t>Clicking Transaction History tab updates URL hash to #direct and shows sub-tabs.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Online sub-tab clickable</t>
+          <t>URL contains #direct; Online and Offline sub-tabs visible</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -3277,12 +3873,12 @@
     <row r="17" ht="55" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TC-4016</t>
+          <t>TC-4014</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Filter Panel Is Visible For Online Payments</t>
+          <t>Offline Payments Sub-tab Is Accessible</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -3292,22 +3888,22 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, online</t>
+          <t>dashboard, pg, sub-tab</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Filter button on Online sub-tab opens filter panel with all time and status options.</t>
+          <t>Offline Payments sub-tab should be visible and clickable.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>All time + status filter options visible</t>
+          <t>Offline sub-tab clickable</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -3325,12 +3921,12 @@
     <row r="18" ht="55" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TC-4017</t>
+          <t>TC-4015</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Filter By All Months For Online Payments</t>
+          <t>Online Payments Sub-tab Is Accessible</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -3340,22 +3936,22 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, online, time-filter</t>
+          <t>dashboard, pg, sub-tab</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>'All Months' time filter option is selectable on Online sub-tab.</t>
+          <t>Online Payments sub-tab should be visible and clickable.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>'All Months' filter selectable</t>
+          <t>Online sub-tab clickable</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -3373,12 +3969,12 @@
     <row r="19" ht="55" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TC-4018</t>
+          <t>TC-4016</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Filter By This Month For Online Payments</t>
+          <t>Filter Panel Is Visible For Online Payments</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3388,22 +3984,22 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, online, time-filter</t>
+          <t>dashboard, pg, filter, online</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>'This Month' time filter option is selectable on Online sub-tab.</t>
+          <t>Filter button on Online sub-tab opens filter panel with all time and status options.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>'This Month' filter selectable</t>
+          <t>All time + status filter options visible</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -3421,12 +4017,12 @@
     <row r="20" ht="55" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TC-4019</t>
+          <t>TC-4017</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Filter By This Year For Online Payments</t>
+          <t>Filter By All Months For Online Payments</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -3446,12 +4042,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>'This Year' time filter option is selectable on Online sub-tab.</t>
+          <t>'All Months' time filter option is selectable on Online sub-tab.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>'This Year' filter selectable</t>
+          <t>'All Months' filter selectable</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -3469,12 +4065,12 @@
     <row r="21" ht="55" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TC-4020</t>
+          <t>TC-4018</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Filter By Last Year For Online Payments</t>
+          <t>Filter By This Month For Online Payments</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -3494,12 +4090,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>'Last Year' time filter option is selectable on Online sub-tab.</t>
+          <t>'This Month' time filter option is selectable on Online sub-tab.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>'Last Year' filter selectable</t>
+          <t>'This Month' filter selectable</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -3517,12 +4113,12 @@
     <row r="22" ht="55" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TC-4021</t>
+          <t>TC-4019</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Filter By Status Paid For Online Payments</t>
+          <t>Filter By This Year For Online Payments</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -3532,7 +4128,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, online, status-filter</t>
+          <t>dashboard, pg, filter, online, time-filter</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -3542,12 +4138,12 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>'Paid' status filter option is selectable on Online sub-tab.</t>
+          <t>'This Year' time filter option is selectable on Online sub-tab.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>'Paid' filter selectable</t>
+          <t>'This Year' filter selectable</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -3565,12 +4161,12 @@
     <row r="23" ht="55" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TC-4022</t>
+          <t>TC-4020</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Filter By Status Failed For Online Payments</t>
+          <t>Filter By Last Year For Online Payments</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -3580,7 +4176,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, online, status-filter</t>
+          <t>dashboard, pg, filter, online, time-filter</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -3590,12 +4186,12 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>'Failed' status filter option is selectable on Online sub-tab.</t>
+          <t>'Last Year' time filter option is selectable on Online sub-tab.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>'Failed' filter selectable</t>
+          <t>'Last Year' filter selectable</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -3613,12 +4209,12 @@
     <row r="24" ht="55" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TC-4023</t>
+          <t>TC-4021</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Filter Panel Is Visible For Offline Payments</t>
+          <t>Filter By Status Paid For Online Payments</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -3628,22 +4224,22 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, offline</t>
+          <t>dashboard, pg, filter, online, status-filter</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Filter button on Offline sub-tab opens filter panel with time filter options only.</t>
+          <t>'Paid' status filter option is selectable on Online sub-tab.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Time filter options visible (no status filters on Offline)</t>
+          <t>'Paid' filter selectable</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -3661,156 +4257,156 @@
     <row r="25" ht="55" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>TC-4022</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Filter By Status Failed For Online Payments</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, pg, filter, online, status-filter</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>'Failed' status filter option is selectable on Online sub-tab.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>'Failed' filter selectable</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>8108556708</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-4023</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Filter Panel Is Visible For Offline Payments</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, pg, filter, offline</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Filter button on Offline sub-tab opens filter panel with time filter options only.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Time filter options visible (no status filters on Offline)</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>8108556708</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="55" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>TC-4024</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Filter By All Months For Offline Payments</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>dashboard, pg, filter, offline, time-filter</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Filter</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>'All Months' time filter is selectable on Offline sub-tab.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>'All Months' filter selectable</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>8108556708</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26" ht="55" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>TC-4025</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Filter By This Month For Offline Payments</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>dashboard, pg, filter, offline, time-filter, robot:skip</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>'This Month' filter for Offline sub-tab.</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>Disabled in Java suite</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="55" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>TC-4026</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Filter By This Year For Offline Payments</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>dashboard, pg, filter, offline, time-filter, robot:skip</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Skipped</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>'This Year' filter for Offline sub-tab.</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>Disabled in Java suite</t>
-        </is>
-      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="55" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TC-4027</t>
+          <t>TC-4025</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Filter By Last Year For Offline Payments</t>
+          <t>Filter By This Month For Offline Payments</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -3830,12 +4426,12 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>'Last Year' time filter is selectable on Offline sub-tab.</t>
+          <t>'This Month' time filter option should be selectable on the Offline sub-tab.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>'Last Year' filter selectable</t>
+          <t>'This Month' filter selectable</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -3853,12 +4449,12 @@
     <row r="29" ht="55" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TC-4028</t>
+          <t>TC-4026</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Clear Filter Button Works</t>
+          <t>Filter By This Year For Offline Payments</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -3868,7 +4464,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, clear-filter</t>
+          <t>dashboard, pg, filter, offline, time-filter</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -3878,12 +4474,12 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>After selecting a filter, clear filter button resets the selection.</t>
+          <t>'This Year' time filter option should be selectable on the Offline sub-tab.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Clear filter button clickable; selection resets</t>
+          <t>'This Year' filter selectable</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -3901,12 +4497,12 @@
     <row r="30" ht="55" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TC-4029</t>
+          <t>TC-4027</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Apply Filter Button Works</t>
+          <t>Filter By Last Year For Offline Payments</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -3916,7 +4512,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, filter, apply-filter</t>
+          <t>dashboard, pg, filter, offline, time-filter</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -3926,12 +4522,12 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>After selecting a filter, apply filter button applies the selection.</t>
+          <t>'Last Year' time filter is selectable on Offline sub-tab.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Apply filter button clickable</t>
+          <t>'Last Year' filter selectable</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -3949,12 +4545,12 @@
     <row r="31" ht="55" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TC-4030</t>
+          <t>TC-4028</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Download Icon Is Visible For Offline Payment</t>
+          <t>Clear Filter Button Works</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -3964,27 +4560,27 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>dashboard, pg, download, offline</t>
+          <t>dashboard, pg, filter, clear-filter</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Download</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Download button for first transaction row on Offline sub-tab should be visible.</t>
+          <t>After selecting a filter, clear filter button resets the selection.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Download button visible on first Offline row</t>
+          <t>Clear filter button clickable; selection resets</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>7757855472 (PG_MOBILE)</t>
+          <t>8108556708</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -3992,59 +4588,155 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Switches to PG_MOBILE via Switch To Account. TC-4031 inherits session.</t>
-        </is>
-      </c>
+      <c r="J31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="55" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>TC-4029</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Apply Filter Button Works</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, pg, filter, apply-filter</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Filter</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>After selecting a filter, apply filter button applies the selection.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Apply filter button clickable</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>8108556708</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33" ht="55" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-4030</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Download Icon Is Visible For Offline Payment</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>dashboard, pg, download, offline</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Download button for first transaction row on Offline sub-tab should be visible.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Download button visible on first Offline row</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>7757855472 (PG_MOBILE)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Switches to PG_MOBILE via Switch To Account. TC-4031 inherits session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="55" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>TC-4031</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Download Icon Is Visible For Online Payment</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>dashboard, pg, download, online</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Download</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Download button for first transaction row on Online sub-tab should be visible.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Download button visible on first Online row</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>Inherits PG_MOBILE session from TC-4030. Canonical from DashboardTestClass3.</t>
         </is>

</xml_diff>

<commit_message>
dashboard and student detail fixes
</commit_message>
<xml_diff>
--- a/CP_UI_Automation_Test_Cases.xlsx
+++ b/CP_UI_Automation_Test_Cases.xlsx
@@ -3430,7 +3430,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard EMI</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8763694182 (AD_MOBILE)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard EMI</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard EMI</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard EMI</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard EMI</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>8763694182 (AD_MOBILE)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>8108556708</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Switches to PG_MOBILE via Switch To Account. TC-4031 inherits session.</t>
+          <t>Independent suite: dashboard_pg_tests.robot uses PG_MOBILE as Suite Setup.</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4990,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Inherits PG_MOBILE session from TC-4030.</t>
+          <t>Independent suite: dashboard_pg_tests.robot.</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>PRECONDITION: AD_MOBILE must have active AD applications. TC-4037–4043 inherit session.</t>
+          <t>Independent suite: dashboard_ad_tests.robot uses AD_MOBILE as Suite Setup. PRECONDITION: AD_MOBILE must have active AD applications.</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard AD</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard New User</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>DASHBOARD_NEW_MOBILE is a dynamically generated fresh mobile. TC-4048–4051 inherit session.</t>
+          <t>Independent suite: dashboard_new_user_tests.robot uses DASHBOARD_NEW_MOBILE as Suite Setup.</t>
         </is>
       </c>
     </row>
@@ -5482,7 +5482,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard New User</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -5530,7 +5530,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard New User</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard New User</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Dashboard PG</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>${DASHBOARD_NEW_MOBILE}</t>
+          <t>7757855472 (PG_MOBILE)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>8108556708 (EXISTING_USER_MOBILE)</t>
+          <t>8108556708 (DASHBOARD_MOBILE)</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>Switches to EXISTING_USER_MOBILE via Switch To Account</t>
+          <t>Runs under DASHBOARD_MOBILE suite session — no Switch To Account needed.</t>
         </is>
       </c>
     </row>
@@ -5861,7 +5861,7 @@
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>Switches to NEW_USER_MOBILE via Switch To Account</t>
+          <t>Switches to NEW_USER_MOBILE within dashboard_tests.robot. TC-4009 (logout) inherits that session.</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Insurance Dashboard</t>
+          <t>Insurance Dashboard New User</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Switches to DASHBOARD_NEW_MOBILE via Navigate To Insurance Tab New User. TC-4113–4115 inherit session.</t>
+          <t>Independent suite: dashboard_ins_new_user_tests.robot uses DASHBOARD_NEW_MOBILE as Suite Setup.</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Insurance Dashboard</t>
+          <t>Insurance Dashboard New User</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -6646,7 +6646,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Insurance Dashboard</t>
+          <t>Insurance Dashboard New User</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6713,7 +6713,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Insurance Dashboard</t>
+          <t>Insurance Dashboard New User</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -6746,7 +6746,7 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6760,7 +6760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7850,6 +7850,689 @@
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TC-5022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>GILE Institute Dropdown Accepts Search And Selects First Option</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Types search term into institute dropdown, waits for async results, and selects the first option using keyboard navigation.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Institute dropdown interaction completes; first option selected</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>9876540001 (APP_CREATION_MOBILE)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>react-select portals menu outside container DOM — uses ArrowDown+Enter with Sleep 2s for async API results</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TC-5023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GILE Location Dropdown Is Selectable After Institute Selection</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>After institute is selected, verifies location dropdown is enabled and first option can be selected.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Location dropdown accepts selection after institute is chosen</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Container click + Sleep 500ms + ArrowDown + Enter (keyboard nav for portalled react-select)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TC-5024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>GILE Board Dropdown Is Selectable After Institute And Location</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>After institute + location are selected, verifies board dropdown is enabled and first option can be selected.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Board dropdown accepts selection</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Container click + Sleep 500ms + ArrowDown + Enter</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TC-5025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Personal Details Section Appears After All GILE Dropdowns Filled</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow, smoke</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Fills all 4 GILE dropdowns in sequence and verifies the personal details section (student-details-title) becomes visible.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>student-details-title visible after all 4 GILE dropdowns filled</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TC-5026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Class Dropdown Is Visible And Selectable After GILE Filled</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Verifies class dropdown is visible and first option is selectable after GILE section is complete.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Class dropdown visible and accepts selection</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TC-5027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Close Button Navigates To Dashboard</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>student-details, application-creation-flow, navigation</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Verifies the Close button on /student-details navigates back to /my-applications. No back-button exists on this page — exit is via data-testid='close-button'.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>URL contains /my-applications after clicking Close</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No back-button on /student-details — uses data-testid='close-button'</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TC-5N-01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Personal Details Section Hidden Before GILE Is Filled</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Verifies student-details-title is not visible on fresh page load before any GILE dropdown is selected.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>student-details-title not visible</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TC-5N-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Show Plans Button Hidden Before GILE Is Filled</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Verifies show-plans-button is not visible before GILE section is complete.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>show-plans-button not visible</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TC-5N-03</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Show Plans With Only First Name Shows Three Errors</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Fills only first name, clicks Show Plans, verifies last name, class, and loan amount errors are shown.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Last name, class, and loan amount validation errors visible</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TC-5N-04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Show Plans With Only Last Name Shows Three Errors</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Fills only last name, clicks Show Plans, verifies first name, class, and loan amount errors are shown.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>First name, class, and loan amount validation errors visible</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>TC-5N-05</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Show Plans With Name Fields Filled But No Class Or Loan Shows Two Errors</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Fills first and last name only, clicks Show Plans, verifies class and loan amount errors are shown.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Class and loan amount validation errors visible</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TC-5N-06</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Show Plans With Name And Class Filled But No Loan Shows Loan Error</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Fills first name, last name, and class, clicks Show Plans, verifies only loan amount error is shown.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Only loan amount validation error visible</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TC-5N-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Show Plans With Only Loan Amount Filled Shows Three Errors</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Fills only loan amount, clicks Show Plans, verifies first name, last name, and class errors are shown.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>First name, last name, and class validation errors visible</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TC-5N-08</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Show Plans With Loan Amount Zero Shows Loan Error</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Student Details</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>student-details, negative</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Fills all required fields with loan amount = 0, clicks Show Plans, verifies loan amount error is shown.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Loan amount validation error visible (0 is invalid)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>9876540001</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Loan amount of 0 triggers validation error — minimum valid amount is &gt; 0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>